<commit_message>
feat(celebrations): per-employee jubilee rules and cake vs flowers
Add celebration_frequency and gift_type on employees and orders, decade/twice-yearly filtering in daily cron, florist 7-day emails, admin/Excel fields, and price_per_flowers on companies.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/happysent-mall.xlsx
+++ b/public/happysent-mall.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>Instruktion (grå rad): Fyll i en rad per person. Födelsedag i formatet ÅÅÅÅ-MM-DD (t.ex. 1992-03-15). Antal personer = hur många kollegor som ska kunna äta tårta den dagen.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+  <si>
+    <t>Instruktion: Fyll i en rad per person. Födelsedag ÅÅÅÅ-MM-DD. Firande (valfritt): varje år | halvår | 10-år. Gåva (valfritt): tårta | blommor.</t>
   </si>
   <si>
     <t>Förnamn</t>
@@ -28,6 +28,12 @@
     <t>Antal personer</t>
   </si>
   <si>
+    <t>Firande</t>
+  </si>
+  <si>
+    <t>Gåva</t>
+  </si>
+  <si>
     <t>Erik</t>
   </si>
   <si>
@@ -37,6 +43,12 @@
     <t>1988-04-22</t>
   </si>
   <si>
+    <t>varje år</t>
+  </si>
+  <si>
+    <t>tårta</t>
+  </si>
+  <si>
     <t>Fatima</t>
   </si>
   <si>
@@ -46,6 +58,12 @@
     <t>1995-11-08</t>
   </si>
   <si>
+    <t>halvår</t>
+  </si>
+  <si>
+    <t>blommor</t>
+  </si>
+  <si>
     <t>Johan</t>
   </si>
   <si>
@@ -53,6 +71,9 @@
   </si>
   <si>
     <t>1990-01-30</t>
+  </si>
+  <si>
+    <t>10-år</t>
   </si>
 </sst>
 </file>
@@ -440,24 +461,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" ht="40" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -470,52 +495,76 @@
       <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D3">
         <v>12</v>
       </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D4">
         <v>8</v>
       </c>
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D5">
         <v>25</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>